<commit_message>
Sept 18 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T2017_GiftLogGiftRequestProcessGiftRequestsVerifyTheTotalsOfTheGiftsAreMeasuredSeparatelyFromTheCurrentYear.xlsx
+++ b/TestData/LV_T2017_GiftLogGiftRequestProcessGiftRequestsVerifyTheTotalsOfTheGiftsAreMeasuredSeparatelyFromTheCurrentYear.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FC2596-5188-48F6-B77C-ACE06BE582F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B09B918-D873-4E28-9C70-0AC50E9DF108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11235" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>

</xml_diff>